<commit_message>
refactor: add schema-driven duplicate detection and validation
- Added Source=key support for duplicate detection
- Updated duplicate check to use schema key row
- Fixed IsMandatory parsing for Excel boolean values
- Replaced hardcoded validation with schema-driven checks
- Updated lookup validation to use LookupMappings InputColumn
- Added validation support for key, filter, lookup and settings sources
- Improved null parent lookup handling
- Verified missing lookup columns fail during validation
- Verified duplicate and failed row handling
</commit_message>
<xml_diff>
--- a/Templates/UsersSchema.xlsx
+++ b/Templates/UsersSchema.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\gitrepos\GMPPro20DataUpload\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDF3766B-7D80-4655-9D1B-B5E14E487700}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFE63B7C-21E5-4D70-8C9A-A58FC9EF2271}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{9A0E982F-1D0A-437F-BDA7-ED9E8C087AEA}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$29</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="69">
   <si>
     <t>Property</t>
   </si>
@@ -63,9 +63,6 @@
     <t>compute</t>
   </si>
   <si>
-    <t>itemID</t>
-  </si>
-  <si>
     <t>flow</t>
   </si>
   <si>
@@ -75,33 +72,18 @@
     <t>publish</t>
   </si>
   <si>
-    <t>designationId</t>
-  </si>
-  <si>
     <t>jsonpath</t>
   </si>
   <si>
-    <t>item</t>
-  </si>
-  <si>
-    <t>displayData</t>
-  </si>
-  <si>
     <t>consume</t>
   </si>
   <si>
     <t>_id</t>
   </si>
   <si>
-    <t>itemCode</t>
-  </si>
-  <si>
     <t>designationCode</t>
   </si>
   <si>
-    <t>designationName</t>
-  </si>
-  <si>
     <t>requestCode</t>
   </si>
   <si>
@@ -117,15 +99,6 @@
     <t>updatedOn</t>
   </si>
   <si>
-    <t>userDetails.designation.itemCode</t>
-  </si>
-  <si>
-    <t>userDetails.designation.item</t>
-  </si>
-  <si>
-    <t>userDetails.designation.displayData</t>
-  </si>
-  <si>
     <t>userDetails.employeeID</t>
   </si>
   <si>
@@ -168,21 +141,6 @@
     <t>usrRequestBasicInfo</t>
   </si>
   <si>
-    <t>masterDesignations</t>
-  </si>
-  <si>
-    <t>designationFormattedName</t>
-  </si>
-  <si>
-    <t>designations.designationCode</t>
-  </si>
-  <si>
-    <t>designations.designationName</t>
-  </si>
-  <si>
-    <t>designations.formattedName</t>
-  </si>
-  <si>
     <t>auto</t>
   </si>
   <si>
@@ -210,9 +168,6 @@
     <t>systemData.moduleCode</t>
   </si>
   <si>
-    <t>userDetails.designation.itemID</t>
-  </si>
-  <si>
     <t>userLoginID</t>
   </si>
   <si>
@@ -240,12 +195,6 @@
     <t>userDetails.officialEmail</t>
   </si>
   <si>
-    <t>itemActualID</t>
-  </si>
-  <si>
-    <t>userDetails.designation.itemActualID</t>
-  </si>
-  <si>
     <t>actualID</t>
   </si>
   <si>
@@ -277,6 +226,15 @@
   </si>
   <si>
     <t>activeStatus</t>
+  </si>
+  <si>
+    <t>userDetails.designation</t>
+  </si>
+  <si>
+    <t>key</t>
+  </si>
+  <si>
+    <t>settings</t>
   </si>
 </sst>
 </file>
@@ -628,7 +586,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2691CE0-5D18-450E-B7A3-EA23A82B1B89}">
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
@@ -657,21 +615,21 @@
         <v>5</v>
       </c>
       <c r="F1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" t="s">
         <v>12</v>
       </c>
-      <c r="G1" t="s">
-        <v>13</v>
-      </c>
       <c r="H1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
@@ -683,21 +641,21 @@
         <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G2" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="H2" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="B3" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -706,30 +664,33 @@
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>68</v>
+      </c>
+      <c r="G3" t="s">
+        <v>44</v>
       </c>
       <c r="H3" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="B4" t="s">
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="G4" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="H4" t="s">
         <v>8</v>
@@ -737,13 +698,13 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="D5" t="b">
         <v>1</v>
@@ -752,15 +713,15 @@
         <v>10</v>
       </c>
       <c r="H5" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
         <v>6</v>
@@ -772,15 +733,15 @@
         <v>10</v>
       </c>
       <c r="H6" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="B7" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
         <v>4</v>
@@ -792,42 +753,42 @@
         <v>10</v>
       </c>
       <c r="H7" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="D8" t="b">
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="F8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G8" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="H8" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" t="s">
         <v>46</v>
       </c>
-      <c r="B9" t="s">
-        <v>22</v>
-      </c>
       <c r="C9" t="s">
         <v>6</v>
       </c>
@@ -835,24 +796,18 @@
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>9</v>
-      </c>
-      <c r="F9" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" t="s">
-        <v>22</v>
+        <v>67</v>
       </c>
       <c r="H9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C10" t="s">
         <v>6</v>
@@ -863,22 +818,16 @@
       <c r="E10" t="s">
         <v>9</v>
       </c>
-      <c r="F10" t="s">
-        <v>14</v>
-      </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>23</v>
-      </c>
-      <c r="H10" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
         <v>6</v>
@@ -887,90 +836,78 @@
         <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F11" t="s">
-        <v>14</v>
-      </c>
-      <c r="G11" t="s">
-        <v>47</v>
+        <v>9</v>
       </c>
       <c r="H11" t="s">
-        <v>50</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="B12" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="C12" t="s">
-        <v>6</v>
+        <v>49</v>
       </c>
       <c r="D12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
       </c>
-      <c r="F12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G12" t="s">
-        <v>24</v>
-      </c>
       <c r="H12" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="C13" t="s">
         <v>6</v>
       </c>
       <c r="D13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H13" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="C14" t="s">
         <v>6</v>
       </c>
       <c r="D14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H14" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="B15" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="C15" t="s">
         <v>6</v>
@@ -982,130 +919,133 @@
         <v>10</v>
       </c>
       <c r="H15" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="C16" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="D16" t="b">
         <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>10</v>
+        <v>59</v>
+      </c>
+      <c r="G16" t="s">
+        <v>17</v>
       </c>
       <c r="H16" t="s">
-        <v>42</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="B17" t="s">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="C17" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="D17" t="b">
         <v>1</v>
       </c>
       <c r="E17" t="s">
-        <v>10</v>
+        <v>59</v>
+      </c>
+      <c r="G17" t="s">
+        <v>58</v>
       </c>
       <c r="H17" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C18" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D18" t="b">
         <v>1</v>
       </c>
       <c r="E18" t="s">
-        <v>10</v>
-      </c>
-      <c r="F18" t="s">
-        <v>19</v>
+        <v>59</v>
       </c>
       <c r="G18" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="H18" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>8</v>
+        <v>63</v>
       </c>
       <c r="C19" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D19" t="b">
         <v>1</v>
       </c>
       <c r="E19" t="s">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="G19" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="H19" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C20" t="s">
-        <v>54</v>
+        <v>6</v>
       </c>
       <c r="D20" t="b">
         <v>1</v>
       </c>
       <c r="E20" t="s">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="F20" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G20" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H20" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="B21" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="C21" t="s">
         <v>6</v>
@@ -1114,21 +1054,24 @@
         <v>1</v>
       </c>
       <c r="E21" t="s">
-        <v>10</v>
+        <v>68</v>
+      </c>
+      <c r="G21" t="s">
+        <v>44</v>
       </c>
       <c r="H21" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="C22" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D22" t="b">
         <v>1</v>
@@ -1137,601 +1080,176 @@
         <v>10</v>
       </c>
       <c r="H22" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>72</v>
+        <v>20</v>
       </c>
       <c r="C23" t="s">
-        <v>54</v>
+        <v>6</v>
       </c>
       <c r="D23" t="b">
         <v>1</v>
       </c>
       <c r="E23" t="s">
-        <v>73</v>
+        <v>10</v>
       </c>
       <c r="H23" t="s">
-        <v>74</v>
+        <v>32</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="C24" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="D24" t="b">
         <v>1</v>
       </c>
       <c r="E24" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H24" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="B25" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="C25" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="D25" t="b">
         <v>1</v>
       </c>
       <c r="E25" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H25" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="B26" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C26" t="s">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="D26" t="b">
         <v>1</v>
       </c>
       <c r="E26" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="F26" t="s">
+        <v>15</v>
+      </c>
+      <c r="G26" t="s">
+        <v>43</v>
       </c>
       <c r="H26" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="B27" t="s">
-        <v>63</v>
+        <v>8</v>
       </c>
       <c r="C27" t="s">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="D27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E27" t="s">
-        <v>10</v>
+        <v>59</v>
+      </c>
+      <c r="G27" t="s">
+        <v>65</v>
       </c>
       <c r="H27" t="s">
-        <v>65</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="B28" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="C28" t="s">
         <v>6</v>
       </c>
       <c r="D28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H28" t="s">
-        <v>67</v>
+        <v>38</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="C29" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E29" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H29" t="s">
-        <v>69</v>
+        <v>39</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>7</v>
+        <v>55</v>
       </c>
       <c r="C30" t="s">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="D30" t="b">
         <v>1</v>
       </c>
       <c r="E30" t="s">
-        <v>10</v>
+        <v>56</v>
       </c>
       <c r="H30" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>37</v>
-      </c>
-      <c r="B31" t="s">
-        <v>11</v>
-      </c>
-      <c r="C31" t="s">
-        <v>6</v>
-      </c>
-      <c r="D31" t="b">
-        <v>1</v>
-      </c>
-      <c r="E31" t="s">
-        <v>10</v>
-      </c>
-      <c r="F31" t="s">
-        <v>19</v>
-      </c>
-      <c r="G31" t="s">
-        <v>15</v>
-      </c>
-      <c r="H31" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
-        <v>37</v>
-      </c>
-      <c r="B32" t="s">
-        <v>70</v>
-      </c>
-      <c r="C32" t="s">
-        <v>6</v>
-      </c>
-      <c r="D32" t="b">
-        <v>1</v>
-      </c>
-      <c r="E32" t="s">
-        <v>10</v>
-      </c>
-      <c r="F32" t="s">
-        <v>19</v>
-      </c>
-      <c r="G32" t="s">
-        <v>15</v>
-      </c>
-      <c r="H32" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>37</v>
-      </c>
-      <c r="B33" t="s">
-        <v>21</v>
-      </c>
-      <c r="C33" t="s">
-        <v>6</v>
-      </c>
-      <c r="D33" t="b">
-        <v>1</v>
-      </c>
-      <c r="E33" t="s">
-        <v>10</v>
-      </c>
-      <c r="F33" t="s">
-        <v>19</v>
-      </c>
-      <c r="G33" t="s">
-        <v>22</v>
-      </c>
-      <c r="H33" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>37</v>
-      </c>
-      <c r="B34" t="s">
-        <v>17</v>
-      </c>
-      <c r="C34" t="s">
-        <v>6</v>
-      </c>
-      <c r="D34" t="b">
-        <v>1</v>
-      </c>
-      <c r="E34" t="s">
-        <v>10</v>
-      </c>
-      <c r="F34" t="s">
-        <v>19</v>
-      </c>
-      <c r="G34" t="s">
-        <v>23</v>
-      </c>
-      <c r="H34" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>37</v>
-      </c>
-      <c r="B35" t="s">
-        <v>18</v>
-      </c>
-      <c r="C35" t="s">
-        <v>6</v>
-      </c>
-      <c r="D35" t="b">
-        <v>1</v>
-      </c>
-      <c r="E35" t="s">
-        <v>10</v>
-      </c>
-      <c r="F35" t="s">
-        <v>19</v>
-      </c>
-      <c r="G35" t="s">
-        <v>47</v>
-      </c>
-      <c r="H35" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
-        <v>37</v>
-      </c>
-      <c r="B36" t="s">
-        <v>75</v>
-      </c>
-      <c r="C36" t="s">
-        <v>64</v>
-      </c>
-      <c r="D36" t="b">
-        <v>1</v>
-      </c>
-      <c r="E36" t="s">
-        <v>76</v>
-      </c>
-      <c r="G36" t="s">
-        <v>75</v>
-      </c>
-      <c r="H36" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
-        <v>37</v>
-      </c>
-      <c r="B37" t="s">
-        <v>78</v>
-      </c>
-      <c r="C37" t="s">
-        <v>64</v>
-      </c>
-      <c r="D37" t="b">
-        <v>1</v>
-      </c>
-      <c r="E37" t="s">
-        <v>76</v>
-      </c>
-      <c r="G37" t="s">
-        <v>78</v>
-      </c>
-      <c r="H37" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
-        <v>37</v>
-      </c>
-      <c r="B38" t="s">
-        <v>80</v>
-      </c>
-      <c r="C38" t="s">
-        <v>64</v>
-      </c>
-      <c r="D38" t="b">
-        <v>1</v>
-      </c>
-      <c r="E38" t="s">
-        <v>76</v>
-      </c>
-      <c r="G38" t="s">
-        <v>80</v>
-      </c>
-      <c r="H38" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
-        <v>37</v>
-      </c>
-      <c r="B39" t="s">
-        <v>24</v>
-      </c>
-      <c r="C39" t="s">
-        <v>6</v>
-      </c>
-      <c r="D39" t="b">
-        <v>1</v>
-      </c>
-      <c r="E39" t="s">
-        <v>10</v>
-      </c>
-      <c r="F39" t="s">
-        <v>19</v>
-      </c>
-      <c r="G39" t="s">
-        <v>24</v>
-      </c>
-      <c r="H39" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
-        <v>37</v>
-      </c>
-      <c r="B40" t="s">
-        <v>58</v>
-      </c>
-      <c r="C40" t="s">
-        <v>6</v>
-      </c>
-      <c r="D40" t="b">
-        <v>1</v>
-      </c>
-      <c r="E40" t="s">
-        <v>10</v>
-      </c>
-      <c r="H40" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
-        <v>37</v>
-      </c>
-      <c r="B41" t="s">
-        <v>25</v>
-      </c>
-      <c r="C41" t="s">
-        <v>6</v>
-      </c>
-      <c r="D41" t="b">
-        <v>1</v>
-      </c>
-      <c r="E41" t="s">
-        <v>10</v>
-      </c>
-      <c r="H41" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
-        <v>37</v>
-      </c>
-      <c r="B42" t="s">
-        <v>26</v>
-      </c>
-      <c r="C42" t="s">
-        <v>6</v>
-      </c>
-      <c r="D42" t="b">
-        <v>1</v>
-      </c>
-      <c r="E42" t="s">
-        <v>10</v>
-      </c>
-      <c r="H42" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
-        <v>37</v>
-      </c>
-      <c r="B43" t="s">
-        <v>27</v>
-      </c>
-      <c r="C43" t="s">
-        <v>38</v>
-      </c>
-      <c r="D43" t="b">
-        <v>1</v>
-      </c>
-      <c r="E43" t="s">
-        <v>10</v>
-      </c>
-      <c r="H43" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>37</v>
-      </c>
-      <c r="B44" t="s">
-        <v>28</v>
-      </c>
-      <c r="C44" t="s">
-        <v>38</v>
-      </c>
-      <c r="D44" t="b">
-        <v>1</v>
-      </c>
-      <c r="E44" t="s">
-        <v>10</v>
-      </c>
-      <c r="H44" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>37</v>
-      </c>
-      <c r="B45" t="s">
-        <v>55</v>
-      </c>
-      <c r="C45" t="s">
-        <v>54</v>
-      </c>
-      <c r="D45" t="b">
-        <v>1</v>
-      </c>
-      <c r="E45" t="s">
-        <v>10</v>
-      </c>
-      <c r="F45" t="s">
-        <v>19</v>
-      </c>
-      <c r="G45" t="s">
         <v>57</v>
-      </c>
-      <c r="H45" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
-        <v>37</v>
-      </c>
-      <c r="B46" t="s">
-        <v>8</v>
-      </c>
-      <c r="C46" t="s">
-        <v>54</v>
-      </c>
-      <c r="D46" t="b">
-        <v>1</v>
-      </c>
-      <c r="E46" t="s">
-        <v>76</v>
-      </c>
-      <c r="G46" t="s">
-        <v>82</v>
-      </c>
-      <c r="H46" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
-        <v>37</v>
-      </c>
-      <c r="B47" t="s">
-        <v>52</v>
-      </c>
-      <c r="C47" t="s">
-        <v>6</v>
-      </c>
-      <c r="D47" t="b">
-        <v>1</v>
-      </c>
-      <c r="E47" t="s">
-        <v>10</v>
-      </c>
-      <c r="H47" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
-        <v>37</v>
-      </c>
-      <c r="B48" t="s">
-        <v>53</v>
-      </c>
-      <c r="C48" t="s">
-        <v>4</v>
-      </c>
-      <c r="D48" t="b">
-        <v>1</v>
-      </c>
-      <c r="E48" t="s">
-        <v>10</v>
-      </c>
-      <c r="H48" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
-        <v>37</v>
-      </c>
-      <c r="B49" t="s">
-        <v>72</v>
-      </c>
-      <c r="C49" t="s">
-        <v>54</v>
-      </c>
-      <c r="D49" t="b">
-        <v>1</v>
-      </c>
-      <c r="E49" t="s">
-        <v>73</v>
-      </c>
-      <c r="H49" t="s">
-        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add schema-driven formula support
- Added Source=formula support in processing framework
- Added Formula column evaluation using placeholder replacement
- Added formula dependency validation
- Added dependency order validation
- Added runtime validation for unresolved placeholders
- Added support for simple formulas such as:
  - {userName} ({employeeID})
  - {designationCode} - {designationName}
  - {departmentCode} - {departmentName}
  - {blockCode} - {blockName}
- Removed hardcoded formattedName generation dependency for schema-based formats
- Verified formula evaluation through user upload testing
- Kept existing compute-based formattedReferenceNumber unchanged
- Kept existing compute-based referenceNumber unchanged
- No formatting specifiers, arithmetic, or conditional expressions in this version
</commit_message>
<xml_diff>
--- a/Templates/UsersSchema.xlsx
+++ b/Templates/UsersSchema.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\gitrepos\GMPPro20DataUpload\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFE63B7C-21E5-4D70-8C9A-A58FC9EF2271}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B217796F-FDAF-4D6D-A773-B151EBD66ED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{9A0E982F-1D0A-437F-BDA7-ED9E8C087AEA}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="71">
   <si>
     <t>Property</t>
   </si>
@@ -235,6 +235,12 @@
   </si>
   <si>
     <t>settings</t>
+  </si>
+  <si>
+    <t>formula</t>
+  </si>
+  <si>
+    <t>{userName} ({employeeID})</t>
   </si>
 </sst>
 </file>
@@ -586,7 +592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2691CE0-5D18-450E-B7A3-EA23A82B1B89}">
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
@@ -598,7 +604,7 @@
     <col min="8" max="8" width="35.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -623,8 +629,11 @@
       <c r="H1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>36</v>
       </c>
@@ -650,7 +659,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>36</v>
       </c>
@@ -673,7 +682,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -696,7 +705,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>36</v>
       </c>
@@ -716,7 +725,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>36</v>
       </c>
@@ -736,7 +745,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>36</v>
       </c>
@@ -756,7 +765,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>36</v>
       </c>
@@ -782,7 +791,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>28</v>
       </c>
@@ -802,7 +811,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>28</v>
       </c>
@@ -822,7 +831,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -842,7 +851,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -862,7 +871,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -882,7 +891,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>28</v>
       </c>
@@ -902,7 +911,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -916,13 +925,16 @@
         <v>1</v>
       </c>
       <c r="E15" t="s">
-        <v>10</v>
+        <v>69</v>
       </c>
       <c r="H15" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I15" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>28</v>
       </c>

</xml_diff>